<commit_message>
Auto commit 01-08-2025 22:45:40.97
</commit_message>
<xml_diff>
--- a/Data Base/Global Templates/150mm Tubewell Construction.xlsx
+++ b/Data Base/Global Templates/150mm Tubewell Construction.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20325"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Core i5 GAMING\Desktop\estimate-drafter\Templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{4FFC6053-6162-4A82-BCDB-1AA54B1A99D3}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19420" windowHeight="11020"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,16 +28,16 @@
     <t>Providing and fixing Bail plug / Bottom plug of required dia to the bottom of pipe assembly of tubewell as per IS : 2800 (part I). 150 mm dia (23.15.2) (Code: GWDDR025)</t>
   </si>
   <si>
-    <t>M.S. cap 150 mm dia (7747 - Water Charge and CPOH Added) (Code: GWDDR024)</t>
-  </si>
-  <si>
     <t>MS Casing pipe 450 mm dia, 6 mm thickness (Code: GWDMR087)</t>
+  </si>
+  <si>
+    <t>PVC End cap 150 mm (DG) (Code: GWDMR004)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -165,7 +159,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -217,7 +211,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -411,21 +405,21 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026E3A80-0F90-4AB8-931D-ABE8CF56B9A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44.28515625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="36.26953125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -433,7 +427,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="120" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="116" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -441,7 +435,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="120" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="116" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -449,7 +443,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="60" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="58" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -457,17 +451,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" ht="29" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="1">
         <v>20</v>

</xml_diff>